<commit_message>
Remover archivos de configuración y excels del rastreo
</commit_message>
<xml_diff>
--- a/salidas_referencia/Boletin_AIOS MENSUAL - copia.xlsx
+++ b/salidas_referencia/Boletin_AIOS MENSUAL - copia.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://superfinanciera-my.sharepoint.com/personal/jemalagon_superfinanciera_gov_co/Documents/ANALITICA PENSIONES/AIOS/para transmision a jun 2025/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\app\plantilla-aios-macro\salidas_referencia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="414" documentId="13_ncr:1_{2F78F793-D0A9-4637-ABD8-C84F07FFB430}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{554A6087-2632-49D8-89DB-E336EE1BEE28}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C70173F-7E82-4524-9CC6-E8A86E9EC98D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="703" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="703" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="3" r:id="rId1"/>
@@ -470,10 +470,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
@@ -763,26 +759,26 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja1"/>
   <dimension ref="A1:S31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.453125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="12.7265625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="11.7265625" style="3" customWidth="1"/>
-    <col min="4" max="4" width="11.54296875" style="3" customWidth="1"/>
+    <col min="1" max="1" width="11.44140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="12.77734375" style="3" customWidth="1"/>
+    <col min="3" max="3" width="11.77734375" style="3" customWidth="1"/>
+    <col min="4" max="4" width="11.5546875" style="3" customWidth="1"/>
     <col min="5" max="5" width="24" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="29.453125" style="3" customWidth="1"/>
-    <col min="7" max="7" width="15.54296875" style="3" customWidth="1"/>
-    <col min="8" max="8" width="16.54296875" style="3" customWidth="1"/>
+    <col min="6" max="6" width="29.44140625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="15.5546875" style="3" customWidth="1"/>
+    <col min="8" max="8" width="16.5546875" style="3" customWidth="1"/>
     <col min="9" max="9" width="24" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="10.7265625" style="3" customWidth="1"/>
-    <col min="12" max="12" width="15.54296875" style="3" customWidth="1"/>
-    <col min="13" max="13" width="13.453125" style="3" customWidth="1"/>
+    <col min="10" max="11" width="10.77734375" style="3" customWidth="1"/>
+    <col min="12" max="12" width="15.5546875" style="3" customWidth="1"/>
+    <col min="13" max="13" width="13.44140625" style="3" customWidth="1"/>
     <col min="14" max="14" width="14" style="3" customWidth="1"/>
-    <col min="15" max="15" width="13.7265625" style="3" customWidth="1"/>
-    <col min="16" max="16" width="18.1796875" style="3" customWidth="1"/>
-    <col min="17" max="17" width="16.54296875" style="3" customWidth="1"/>
-    <col min="18" max="18" width="18.1796875" style="3" customWidth="1"/>
-    <col min="19" max="16384" width="10.7265625" style="3"/>
+    <col min="15" max="15" width="13.77734375" style="3" customWidth="1"/>
+    <col min="16" max="16" width="18.21875" style="3" customWidth="1"/>
+    <col min="17" max="17" width="16.5546875" style="3" customWidth="1"/>
+    <col min="18" max="18" width="18.21875" style="3" customWidth="1"/>
+    <col min="19" max="16384" width="10.77734375" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" s="1" customFormat="1" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -844,7 +840,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>45108</v>
       </c>
@@ -903,7 +899,7 @@
         <v>3923.49</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>45139</v>
       </c>
@@ -962,7 +958,7 @@
         <v>4085.33</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>45170</v>
       </c>
@@ -1021,7 +1017,7 @@
         <v>4053.76</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>45200</v>
       </c>
@@ -1080,7 +1076,7 @@
         <v>4060.83</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>45231</v>
       </c>
@@ -1139,7 +1135,7 @@
         <v>3980.67</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>45261</v>
       </c>
@@ -1198,7 +1194,7 @@
         <v>3822.05</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>45292</v>
       </c>
@@ -1257,7 +1253,7 @@
         <v>3925.6</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>45323</v>
       </c>
@@ -1316,7 +1312,7 @@
         <v>3933.56</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>45352</v>
       </c>
@@ -1375,7 +1371,7 @@
         <v>3842.3</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>45383</v>
       </c>
@@ -1434,7 +1430,7 @@
         <v>3873.44</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>45413</v>
       </c>
@@ -1493,7 +1489,7 @@
         <v>3874.32</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>45444</v>
       </c>
@@ -1552,7 +1548,7 @@
         <v>4148.04</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>45474</v>
       </c>
@@ -1611,7 +1607,7 @@
         <v>4089.05</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>45505</v>
       </c>
@@ -1670,7 +1666,7 @@
         <v>4160.3100000000004</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>45536</v>
       </c>
@@ -1729,7 +1725,7 @@
         <v>4164.21</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>45566</v>
       </c>
@@ -1788,7 +1784,7 @@
         <v>4413.46</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>45597</v>
       </c>
@@ -1847,7 +1843,7 @@
         <v>4419.59</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>45627</v>
       </c>
@@ -1906,7 +1902,7 @@
         <v>4409.1499999999996</v>
       </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>45658</v>
       </c>
@@ -1965,7 +1961,7 @@
         <v>4170.01</v>
       </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>45689</v>
       </c>
@@ -2024,7 +2020,7 @@
         <v>4120.1099999999997</v>
       </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>45717</v>
       </c>
@@ -2083,7 +2079,7 @@
         <v>4192.57</v>
       </c>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>45748</v>
       </c>
@@ -2142,7 +2138,7 @@
         <v>4198.83</v>
       </c>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>45778</v>
       </c>
@@ -2201,7 +2197,7 @@
         <v>4148.72</v>
       </c>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>45809</v>
       </c>
@@ -2260,26 +2256,29 @@
         <v>4069.67</v>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:19" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A26" s="2">
+        <v>45839</v>
+      </c>
       <c r="F26" s="22"/>
       <c r="G26" s="23"/>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.3">
       <c r="F27"/>
       <c r="G27"/>
       <c r="N27" s="31"/>
       <c r="O27" s="31"/>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.3">
       <c r="F28" s="20"/>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.3">
       <c r="F29" s="20"/>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.3">
       <c r="F30" s="20"/>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.3">
       <c r="G31" s="21"/>
     </row>
   </sheetData>

</xml_diff>